<commit_message>
Heladería EN ronda 1: los 11 xlsx remontados (gates VERDE 8/0, autotest 19/19, 0 celdas cortadas nuevas)
Textos, censo y pendientes regenerados tras el parche del ES (87 heredadas, 403 pendientes = G1). gates_en.py:
«dulce de leche» en FRASES_OK (G2 lo leía como español); los 7 kits publicados dan la misma salida que con el
gates_en de main. censo-entregables 0 y no-latinos 0 (EN y ES); sha256 VPS = Mac; volcados nuevos.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Via: Claude Code
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/ice-cream-shop-checklist-templates/01-ice-cream-shop-opening-closing-checklists.xlsx
+++ b/astro-site/public/dl/ice-cream-shop-checklist-templates/01-ice-cream-shop-opening-closing-checklists.xlsx
@@ -648,9 +648,9 @@
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="24" t="inlineStr">
-        <is>
-          <t>▸ Includes switching the dipping cabinets to service mode, walk-in checks, setup and closing.</t>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>▸ Includes the dipping cabinet and walk-in checks, setup and closing.</t>
         </is>
       </c>
     </row>
@@ -706,14 +706,14 @@
     <row r="16">
       <c r="B16" s="24" t="inlineStr">
         <is>
-          <t>▸ A shop runs three different temperatures; never mix them up: storage 0 °F or below, dipping cabinet service 6–10 °F (per the manufacturer) and mix aging 36–39 °F, never above 41 °F. Dipping cabinets are NOT turned off at night: they go to storage mode.</t>
+          <t>▸ A shop runs three different temperatures; never mix them up: storage 0 °F or below, dipping cabinet service 6–10 °F (per the manufacturer) and mix aging 36–39 °F, never above 41 °F. Dipping cabinets are NOT turned off at night: they stay on — on their night/storage setting if your model has one, per the manufacturer.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="24" t="inlineStr">
         <is>
-          <t>▸ Allergens travel on the scoop: use the dipper well or one scoop per flavor. Water does not remove allergens: for an allergy order, wash hands, wear fresh gloves and use a clean, sanitized scoop. Cones, wafers and cookies contain wheat; pistachio, hazelnut and almond are tree nuts (US: 9 major allergens; UK: 14).</t>
+          <t>▸ Allergens travel on the scoop: use the dipper well or one scoop per flavor. Water does not remove allergens: for an allergy order, wash hands, wear fresh gloves and use a clean, sanitized scoop. Cones, wafers and cookies contain wheat; pistachio, hazelnut and almond are tree nuts, and peanut butter flavors and toppings carry peanuts (US: 9 major allergens; UK: 14).</t>
         </is>
       </c>
     </row>
@@ -942,7 +942,7 @@
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>If the production room or waffle/crepe area has GAS: open the main valve and check there is NO gas smell BEFORE turning anything on. If you smell gas, touch nothing, get everyone out and call the gas company or 911 from outside</t>
+          <t>If the production room or waffle/crepe area has GAS: check there is NO gas smell BEFORE lighting anything. If you smell gas, touch nothing, get everyone out and call the gas company or 911 from outside</t>
         </is>
       </c>
       <c r="C12" s="22" t="inlineStr">
@@ -1008,7 +1008,7 @@
       </c>
       <c r="B16" s="9" t="inlineStr">
         <is>
-          <t>Switch the dipping cabinets from overnight storage (0 °F) to service mode (6–10 °F, per the manufacturer) and confirm they held temperature all night — log reading: ____ °F</t>
+          <t>First thing: if your dipping cabinets have a night/storage setting, switch them back to service mode (6–10 °F, per the manufacturer), and confirm they held temperature all night — log reading: ____ °F</t>
         </is>
       </c>
       <c r="C16" s="10" t="inlineStr">
@@ -1046,7 +1046,7 @@
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t>Check the aging cooler (36–39 °F) — log reading: ____ °F: above 41 °F the pasteurized mix is no longer safe</t>
+          <t>Check the aging cooler (36–39 °F) — log reading: ____ °F: above 41 °F, the person in charge assesses the mix (how warm, for how long) before it is used</t>
         </is>
       </c>
       <c r="C18" s="14" t="inlineStr">
@@ -1185,7 +1185,7 @@
       </c>
       <c r="B26" s="9" t="inlineStr">
         <is>
-          <t>Use the dipper well (running water) or one scoop per flavor: tree nuts (pistachio, hazelnut, almond) travel from pan to pan on the scoop</t>
+          <t>Use the dipper well (running water) or one scoop per flavor: tree nuts and peanuts (pistachio, hazelnut, peanut butter) travel from pan to pan on the scoop</t>
         </is>
       </c>
       <c r="C26" s="16" t="inlineStr">
@@ -1223,7 +1223,7 @@
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>Prepare sauces: chocolate, caramel, berry, milk caramel (dairy and cut fruit covered at 41 °F or below; hot fudge in its warmer per the manufacturer)</t>
+          <t>Prepare sauces: chocolate, caramel, berry, dulce de leche (dairy and cut fruit covered at 41 °F or below; hot fudge in its warmer per the manufacturer)</t>
         </is>
       </c>
       <c r="C28" s="16" t="inlineStr">
@@ -1621,7 +1621,7 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>Switch the dipping cabinets to storage mode (0 °F): never turn them off — with product inside, an overnight shutdown can ruin the whole batch</t>
+          <t>Leave the dipping cabinets ON (never turn them off with product inside: an overnight shutdown can ruin the whole batch); use the night/storage setting only if your model has one, per the manufacturer</t>
         </is>
       </c>
       <c r="C7" s="10" t="inlineStr">

</xml_diff>